<commit_message>
chore: update SEFAZ ICMS-SP data through April 2026
Pipeline run 20260423-071136 ratifies the data:
- 280 observations (2003-01 → 2026-04)
- realized YTD 2026: R$ 78,2 bi (jan+fev+mar+abr)
- ensemble 2026 forecast: R$ 246,0 bi (IC95% 240,6–251,7)
- best model: Ensemble(M1,M2,M3,M4), MAPE 1,92%
- 9/9 models fitted, 4/5 validation checks pass (Ljung-Box warn known)
</commit_message>
<xml_diff>
--- a/data/dados_sefaz.xlsx
+++ b/data/dados_sefaz.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fazendaspgovbr-my.sharepoint.com/personal/blzulian_fazenda_sp_gov_br/Documents/Documentos/Assessoria/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\linuxadmin\repos\engine-DAGs\previsao-icms-sp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D075434-71AB-451F-9A46-C2A563FF8471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46FB318-4ED3-4247-B0B7-D7062E1EC054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D1BA120B-327D-4E8F-B505-62329AFF60E5}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="28800" windowHeight="15285" xr2:uid="{D1BA120B-327D-4E8F-B505-62329AFF60E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -734,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A331E3F-F37F-4C01-AD6B-8C59340D4B1D}">
-  <dimension ref="A1:B280"/>
+  <dimension ref="A1:B281"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -3003,8 +3003,16 @@
         <v>46082</v>
       </c>
       <c r="B280" s="3">
-        <f>14700.3466276187/0.75*10^6</f>
-        <v>19600462170.158264</v>
+        <v>19607474765.560001</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A281" s="2">
+        <v>46113</v>
+      </c>
+      <c r="B281" s="3">
+        <f>15073/0.75*10^6</f>
+        <v>20097333333.333332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>